<commit_message>
feat: created accept/reject PRNs page
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
+++ b/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="49">
   <si>
     <t>Translator notes</t>
   </si>
@@ -46,10 +46,10 @@
     <t>producer-prns-list</t>
   </si>
   <si>
-    <t>Multiple PRN/PERN list page for producer.</t>
-  </si>
-  <si>
-    <t>PRNs and PERNs</t>
+    <t>Accept/reject awaiting-acceptance PRN/PERN list for producer (MO-427).</t>
+  </si>
+  <si>
+    <t>Accept or reject PRNs and PERNs</t>
   </si>
   <si>
     <t/>
@@ -58,37 +58,64 @@
     <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-113376&amp;t=kGagF0SHsPR8Aw1a-4</t>
   </si>
   <si>
+    <t>prns.list.intro</t>
+  </si>
+  <si>
+    <t>Select the PRNs or PERNs you want to accept. You can also review each one by opening it and selecting 'accept' or 'reject'.</t>
+  </si>
+  <si>
     <t>prns.list.resultsSummary</t>
   </si>
   <si>
-    <t>Showing {{count}} of {{total}}</t>
+    <t>Showing {{from}} to {{to}} of {{total}}</t>
   </si>
   <si>
     <t>prns.list.noPrnsFound</t>
   </si>
   <si>
-    <t>No PRNs or PERNs were found for this organisation.</t>
+    <t>You have no PRNs or PERNs awaiting acceptance.</t>
+  </si>
+  <si>
+    <t>prns.list.acceptSelectedButton</t>
+  </si>
+  <si>
+    <t>Accept selected PRNs and PERNs</t>
+  </si>
+  <si>
+    <t>prns.list.notProvided</t>
+  </si>
+  <si>
+    <t>Not provided</t>
+  </si>
+  <si>
+    <t>prns.list.yes</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>prns.list.no</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>prns.list.selectPrnHiddenText</t>
+  </si>
+  <si>
+    <t>Select {{number}}</t>
+  </si>
+  <si>
+    <t>prns.list.tableCaption</t>
+  </si>
+  <si>
+    <t>A list of PRNs and PERNs to select from.</t>
   </si>
   <si>
     <t>prns.list.table.number</t>
   </si>
   <si>
-    <t>Number</t>
-  </si>
-  <si>
-    <t>prns.list.table.type</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>prns.list.table.status</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Statws</t>
+    <t>PRN or PERN number</t>
   </si>
   <si>
     <t>prns.list.table.material</t>
@@ -100,6 +127,24 @@
     <t>Deunydd</t>
   </si>
   <si>
+    <t>prns.list.table.issuedAt</t>
+  </si>
+  <si>
+    <t>Date issued</t>
+  </si>
+  <si>
+    <t>prns.list.table.decemberWaste</t>
+  </si>
+  <si>
+    <t>December waste</t>
+  </si>
+  <si>
+    <t>prns.list.table.issuer</t>
+  </si>
+  <si>
+    <t>Issued by</t>
+  </si>
+  <si>
     <t>prns.list.table.tonnage</t>
   </si>
   <si>
@@ -109,28 +154,10 @@
     <t>Tunelli</t>
   </si>
   <si>
-    <t>prns.list.table.issuedAt</t>
-  </si>
-  <si>
-    <t>Date issued</t>
-  </si>
-  <si>
-    <t>prns.list.table.issuer</t>
-  </si>
-  <si>
-    <t>Issuer</t>
-  </si>
-  <si>
-    <t>prns.list.table.view</t>
-  </si>
-  <si>
-    <t>View</t>
-  </si>
-  <si>
-    <t>prns.list.table.viewHiddenText</t>
-  </si>
-  <si>
-    <t>View {{number}}</t>
+    <t>prns.list.table.issuerNote</t>
+  </si>
+  <si>
+    <t>Issuer note</t>
   </si>
 </sst>
 </file>
@@ -529,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -600,7 +627,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -694,7 +721,7 @@
         <v>24</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>13</v>
@@ -702,19 +729,19 @@
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="E12" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>13</v>
@@ -722,7 +749,7 @@
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>10</v>
@@ -731,10 +758,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>13</v>
@@ -742,7 +769,7 @@
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>10</v>
@@ -751,7 +778,7 @@
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>13</v>
@@ -762,7 +789,7 @@
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>10</v>
@@ -771,7 +798,7 @@
         <v>11</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>13</v>
@@ -782,7 +809,7 @@
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>10</v>
@@ -791,7 +818,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>13</v>
@@ -802,26 +829,126 @@
     </row>
     <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="1" t="s">
+      <c r="B18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="1" t="s">
+      <c r="E18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F17"/>
+  <autoFilter ref="A5:F22"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
feat: MO-428 Add sort/filterby by options to PRN/PERN list
- fix translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
+++ b/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="113">
   <si>
     <t>Translator notes</t>
   </si>
@@ -19,7 +19,7 @@
     <t>Translations with syntax such as {{year}} should be preserved in the translated text, as it's a placeholder for a dynamic value</t>
   </si>
   <si>
-    <t>Reusable content rendered on this page is translated in: 00-shared-layout.xlsx.</t>
+    <t>Reusable content rendered on this page is translated in: 00-shared-layout.xlsx, 07-producer-certificate-submit.xlsx.</t>
   </si>
   <si>
     <t>Translation key</t>
@@ -46,7 +46,7 @@
     <t>producer-prns-list</t>
   </si>
   <si>
-    <t>Accept/reject awaiting-acceptance PRN/PERN list for producer (MO-427).</t>
+    <t>Multiple PRN/PERN list page for producer, including the error summary when accept selected is submitted with no checkboxes.</t>
   </si>
   <si>
     <t>Accept or reject PRNs and PERNs</t>
@@ -55,7 +55,13 @@
     <t/>
   </si>
   <si>
-    <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-113376&amp;t=kGagF0SHsPR8Aw1a-4</t>
+    <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=3481-100802&amp;t=NRZGtCe2tBGc3HxG-4</t>
+  </si>
+  <si>
+    <t>prns.list.pageHeadingForYear</t>
+  </si>
+  <si>
+    <t>Accept or reject PRNs and PERNs for {{year}}</t>
   </si>
   <si>
     <t>prns.list.intro</t>
@@ -112,6 +118,42 @@
     <t>A list of PRNs and PERNs to select from.</t>
   </si>
   <si>
+    <t>prns.list.sortBy</t>
+  </si>
+  <si>
+    <t>Sort by</t>
+  </si>
+  <si>
+    <t>Didoli yn ôl</t>
+  </si>
+  <si>
+    <t>prns.list.filterBy</t>
+  </si>
+  <si>
+    <t>Filter by</t>
+  </si>
+  <si>
+    <t>Hidlo yn ol</t>
+  </si>
+  <si>
+    <t>prns.list.applyFilter</t>
+  </si>
+  <si>
+    <t>Apply</t>
+  </si>
+  <si>
+    <t>Cymhwyso</t>
+  </si>
+  <si>
+    <t>prns.list.clearAll</t>
+  </si>
+  <si>
+    <t>Clear all</t>
+  </si>
+  <si>
+    <t>Clirio'r cyfan</t>
+  </si>
+  <si>
     <t>prns.list.table.number</t>
   </si>
   <si>
@@ -158,6 +200,156 @@
   </si>
   <si>
     <t>Issuer note</t>
+  </si>
+  <si>
+    <t>prns.list.errors.selectOneOrMore</t>
+  </si>
+  <si>
+    <t>To accept multiple PRNs or PERNs select one or more using the check boxes</t>
+  </si>
+  <si>
+    <t>prns.list.sort.issuedAtDescending</t>
+  </si>
+  <si>
+    <t>Date issued (newest first)</t>
+  </si>
+  <si>
+    <t>Dyddiad rhoi (diweddaraf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.issuedAtAscending</t>
+  </si>
+  <si>
+    <t>Date issued (oldest first)</t>
+  </si>
+  <si>
+    <t>Dyddiad rhoi (hynaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.materialAscending</t>
+  </si>
+  <si>
+    <t>Material by (A to Z)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.materialDescending</t>
+  </si>
+  <si>
+    <t>Material by (Z to A)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.tonnageDescending</t>
+  </si>
+  <si>
+    <t>Tonnage: (heaviest first)</t>
+  </si>
+  <si>
+    <t>Tunelli (trymaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.tonnageAscending</t>
+  </si>
+  <si>
+    <t>Tonnage: (lightest first)</t>
+  </si>
+  <si>
+    <t>Tunelli (ysgafnaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.filter.all</t>
+  </si>
+  <si>
+    <t>All materials</t>
+  </si>
+  <si>
+    <t>Pob deunydd</t>
+  </si>
+  <si>
+    <t>prns.list.filter.aluminium</t>
+  </si>
+  <si>
+    <t>Aluminium</t>
+  </si>
+  <si>
+    <t>Alwminiwm</t>
+  </si>
+  <si>
+    <t>prns.list.filter.glassOther</t>
+  </si>
+  <si>
+    <t>Glass other</t>
+  </si>
+  <si>
+    <t>Gwydr arall</t>
+  </si>
+  <si>
+    <t>prns.list.filter.glassRemelt</t>
+  </si>
+  <si>
+    <t>Glass re-melt</t>
+  </si>
+  <si>
+    <t>Gwydr aildoddi</t>
+  </si>
+  <si>
+    <t>prns.list.filter.paper</t>
+  </si>
+  <si>
+    <t>Paper, board or fibre-based composite material</t>
+  </si>
+  <si>
+    <t>Papur, bwrdd neu ddeunydd cyfansawdd sy'n seiliedig ar ffeibrau</t>
+  </si>
+  <si>
+    <t>prns.list.filter.plastic</t>
+  </si>
+  <si>
+    <t>Plastic</t>
+  </si>
+  <si>
+    <t>Plastig</t>
+  </si>
+  <si>
+    <t>prns.list.filter.steel</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>Dur</t>
+  </si>
+  <si>
+    <t>prns.list.filter.wood</t>
+  </si>
+  <si>
+    <t>Wood</t>
+  </si>
+  <si>
+    <t>Pren</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.landmark</t>
+  </si>
+  <si>
+    <t>results</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.previous</t>
+  </si>
+  <si>
+    <t>Previous</t>
+  </si>
+  <si>
+    <t>Blaenorol</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.next</t>
+  </si>
+  <si>
+    <t>Next</t>
+  </si>
+  <si>
+    <t>Nesaf</t>
   </si>
 </sst>
 </file>
@@ -556,7 +748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -627,7 +819,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -647,7 +839,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -861,7 +1053,7 @@
         <v>39</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>13</v>
@@ -869,7 +1061,7 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>10</v>
@@ -878,10 +1070,10 @@
         <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>13</v>
@@ -889,7 +1081,7 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>10</v>
@@ -898,10 +1090,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>13</v>
@@ -909,7 +1101,7 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>10</v>
@@ -918,10 +1110,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
@@ -929,7 +1121,7 @@
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>10</v>
@@ -938,17 +1130,477 @@
         <v>11</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F22"/>
+  <autoFilter ref="A5:F45"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
feat: MO-428 Add sort/filterby options to PRN/PERN list
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
+++ b/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="113">
   <si>
     <t>Translator notes</t>
   </si>
@@ -19,7 +19,7 @@
     <t>Translations with syntax such as {{year}} should be preserved in the translated text, as it's a placeholder for a dynamic value</t>
   </si>
   <si>
-    <t>Reusable content rendered on this page is translated in: 00-shared-layout.xlsx.</t>
+    <t>Reusable content rendered on this page is translated in: 00-shared-layout.xlsx, 07-producer-certificate-submit.xlsx.</t>
   </si>
   <si>
     <t>Translation key</t>
@@ -46,7 +46,7 @@
     <t>producer-prns-list</t>
   </si>
   <si>
-    <t>Accept/reject awaiting-acceptance PRN/PERN list for producer (MO-427).</t>
+    <t>Multiple PRN/PERN list page for producer, including the error summary when accept selected is submitted with no checkboxes.</t>
   </si>
   <si>
     <t>Accept or reject PRNs and PERNs</t>
@@ -55,7 +55,13 @@
     <t/>
   </si>
   <si>
-    <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-113376&amp;t=kGagF0SHsPR8Aw1a-4</t>
+    <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=3481-100802&amp;t=NRZGtCe2tBGc3HxG-4</t>
+  </si>
+  <si>
+    <t>prns.list.pageHeadingForYear</t>
+  </si>
+  <si>
+    <t>Accept or reject PRNs and PERNs for {{year}}</t>
   </si>
   <si>
     <t>prns.list.intro</t>
@@ -112,6 +118,42 @@
     <t>A list of PRNs and PERNs to select from.</t>
   </si>
   <si>
+    <t>prns.list.sortBy</t>
+  </si>
+  <si>
+    <t>Sort by</t>
+  </si>
+  <si>
+    <t>Didoli yn ôl</t>
+  </si>
+  <si>
+    <t>prns.list.filterBy</t>
+  </si>
+  <si>
+    <t>Filter by</t>
+  </si>
+  <si>
+    <t>Hidlo yn ol</t>
+  </si>
+  <si>
+    <t>prns.list.applyFilter</t>
+  </si>
+  <si>
+    <t>Apply</t>
+  </si>
+  <si>
+    <t>Cymhwyso</t>
+  </si>
+  <si>
+    <t>prns.list.clearAll</t>
+  </si>
+  <si>
+    <t>Clear all</t>
+  </si>
+  <si>
+    <t>Clirio'r cyfan</t>
+  </si>
+  <si>
     <t>prns.list.table.number</t>
   </si>
   <si>
@@ -158,6 +200,156 @@
   </si>
   <si>
     <t>Issuer note</t>
+  </si>
+  <si>
+    <t>prns.list.errors.selectOneOrMore</t>
+  </si>
+  <si>
+    <t>To accept multiple PRNs or PERNs select one or more using the check boxes</t>
+  </si>
+  <si>
+    <t>prns.list.sort.issuedAtDescending</t>
+  </si>
+  <si>
+    <t>Date issued (newest first)</t>
+  </si>
+  <si>
+    <t>Dyddiad rhoi (diweddaraf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.issuedAtAscending</t>
+  </si>
+  <si>
+    <t>Date issued (oldest first)</t>
+  </si>
+  <si>
+    <t>Dyddiad rhoi (hynaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.materialAscending</t>
+  </si>
+  <si>
+    <t>Material by (A to Z)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.materialDescending</t>
+  </si>
+  <si>
+    <t>Material by (Z to A)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.tonnageDescending</t>
+  </si>
+  <si>
+    <t>Tonnage: (heaviest first)</t>
+  </si>
+  <si>
+    <t>Tunelli (trymaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.tonnageAscending</t>
+  </si>
+  <si>
+    <t>Tonnage: (lightest first)</t>
+  </si>
+  <si>
+    <t>Tunelli (ysgafnaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.filter.all</t>
+  </si>
+  <si>
+    <t>All materials</t>
+  </si>
+  <si>
+    <t>Pob deunydd</t>
+  </si>
+  <si>
+    <t>prns.list.filter.aluminium</t>
+  </si>
+  <si>
+    <t>Aluminium</t>
+  </si>
+  <si>
+    <t>Alwminiwm</t>
+  </si>
+  <si>
+    <t>prns.list.filter.glassOther</t>
+  </si>
+  <si>
+    <t>Glass other</t>
+  </si>
+  <si>
+    <t>Gwydr arall</t>
+  </si>
+  <si>
+    <t>prns.list.filter.glassRemelt</t>
+  </si>
+  <si>
+    <t>Glass re-melt</t>
+  </si>
+  <si>
+    <t>Gwydr aildoddi</t>
+  </si>
+  <si>
+    <t>prns.list.filter.paper</t>
+  </si>
+  <si>
+    <t>Paper, board or fibre-based composite material</t>
+  </si>
+  <si>
+    <t>Papur, bwrdd neu ddeunydd cyfansawdd sy'n seiliedig ar ffeibrau</t>
+  </si>
+  <si>
+    <t>prns.list.filter.plastic</t>
+  </si>
+  <si>
+    <t>Plastic</t>
+  </si>
+  <si>
+    <t>Plastig</t>
+  </si>
+  <si>
+    <t>prns.list.filter.steel</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>Dur</t>
+  </si>
+  <si>
+    <t>prns.list.filter.wood</t>
+  </si>
+  <si>
+    <t>Wood</t>
+  </si>
+  <si>
+    <t>Pren</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.landmark</t>
+  </si>
+  <si>
+    <t>results</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.previous</t>
+  </si>
+  <si>
+    <t>Previous</t>
+  </si>
+  <si>
+    <t>Blaenorol</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.next</t>
+  </si>
+  <si>
+    <t>Next</t>
+  </si>
+  <si>
+    <t>Nesaf</t>
   </si>
 </sst>
 </file>
@@ -556,7 +748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -627,7 +819,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -647,7 +839,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -861,7 +1053,7 @@
         <v>39</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>13</v>
@@ -869,7 +1061,7 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>10</v>
@@ -878,10 +1070,10 @@
         <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>13</v>
@@ -889,7 +1081,7 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>10</v>
@@ -898,10 +1090,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>13</v>
@@ -909,7 +1101,7 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>10</v>
@@ -918,10 +1110,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
@@ -929,7 +1121,7 @@
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>10</v>
@@ -938,17 +1130,477 @@
         <v>11</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F22"/>
+  <autoFilter ref="A5:F45"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
Feat/428 accept reject filters (#174)
* feat: MO-428 Add sort/filterby options to PRN/PERN list

* Fix lock file
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
+++ b/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="113">
   <si>
     <t>Translator notes</t>
   </si>
@@ -19,7 +19,7 @@
     <t>Translations with syntax such as {{year}} should be preserved in the translated text, as it's a placeholder for a dynamic value</t>
   </si>
   <si>
-    <t>Reusable content rendered on this page is translated in: 00-shared-layout.xlsx.</t>
+    <t>Reusable content rendered on this page is translated in: 00-shared-layout.xlsx, 07-producer-certificate-submit.xlsx.</t>
   </si>
   <si>
     <t>Translation key</t>
@@ -46,7 +46,7 @@
     <t>producer-prns-list</t>
   </si>
   <si>
-    <t>Accept/reject awaiting-acceptance PRN/PERN list for producer (MO-427).</t>
+    <t>Multiple PRN/PERN list page for producer, including the error summary when accept selected is submitted with no checkboxes.</t>
   </si>
   <si>
     <t>Accept or reject PRNs and PERNs</t>
@@ -55,7 +55,13 @@
     <t/>
   </si>
   <si>
-    <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=1915-113376&amp;t=kGagF0SHsPR8Aw1a-4</t>
+    <t>https://www.figma.com/design/T6jnQSPgRrAAYGSykX5Fca/Multi-year-and-Dec-Waste?node-id=3481-100802&amp;t=NRZGtCe2tBGc3HxG-4</t>
+  </si>
+  <si>
+    <t>prns.list.pageHeadingForYear</t>
+  </si>
+  <si>
+    <t>Accept or reject PRNs and PERNs for {{year}}</t>
   </si>
   <si>
     <t>prns.list.intro</t>
@@ -112,6 +118,42 @@
     <t>A list of PRNs and PERNs to select from.</t>
   </si>
   <si>
+    <t>prns.list.sortBy</t>
+  </si>
+  <si>
+    <t>Sort by</t>
+  </si>
+  <si>
+    <t>Didoli yn ôl</t>
+  </si>
+  <si>
+    <t>prns.list.filterBy</t>
+  </si>
+  <si>
+    <t>Filter by</t>
+  </si>
+  <si>
+    <t>Hidlo yn ol</t>
+  </si>
+  <si>
+    <t>prns.list.applyFilter</t>
+  </si>
+  <si>
+    <t>Apply</t>
+  </si>
+  <si>
+    <t>Cymhwyso</t>
+  </si>
+  <si>
+    <t>prns.list.clearAll</t>
+  </si>
+  <si>
+    <t>Clear all</t>
+  </si>
+  <si>
+    <t>Clirio'r cyfan</t>
+  </si>
+  <si>
     <t>prns.list.table.number</t>
   </si>
   <si>
@@ -158,6 +200,156 @@
   </si>
   <si>
     <t>Issuer note</t>
+  </si>
+  <si>
+    <t>prns.list.errors.selectOneOrMore</t>
+  </si>
+  <si>
+    <t>To accept multiple PRNs or PERNs select one or more using the check boxes</t>
+  </si>
+  <si>
+    <t>prns.list.sort.issuedAtDescending</t>
+  </si>
+  <si>
+    <t>Date issued (newest first)</t>
+  </si>
+  <si>
+    <t>Dyddiad rhoi (diweddaraf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.issuedAtAscending</t>
+  </si>
+  <si>
+    <t>Date issued (oldest first)</t>
+  </si>
+  <si>
+    <t>Dyddiad rhoi (hynaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.materialAscending</t>
+  </si>
+  <si>
+    <t>Material by (A to Z)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.materialDescending</t>
+  </si>
+  <si>
+    <t>Material by (Z to A)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.tonnageDescending</t>
+  </si>
+  <si>
+    <t>Tonnage: (heaviest first)</t>
+  </si>
+  <si>
+    <t>Tunelli (trymaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.sort.tonnageAscending</t>
+  </si>
+  <si>
+    <t>Tonnage: (lightest first)</t>
+  </si>
+  <si>
+    <t>Tunelli (ysgafnaf yn gyntaf)</t>
+  </si>
+  <si>
+    <t>prns.list.filter.all</t>
+  </si>
+  <si>
+    <t>All materials</t>
+  </si>
+  <si>
+    <t>Pob deunydd</t>
+  </si>
+  <si>
+    <t>prns.list.filter.aluminium</t>
+  </si>
+  <si>
+    <t>Aluminium</t>
+  </si>
+  <si>
+    <t>Alwminiwm</t>
+  </si>
+  <si>
+    <t>prns.list.filter.glassOther</t>
+  </si>
+  <si>
+    <t>Glass other</t>
+  </si>
+  <si>
+    <t>Gwydr arall</t>
+  </si>
+  <si>
+    <t>prns.list.filter.glassRemelt</t>
+  </si>
+  <si>
+    <t>Glass re-melt</t>
+  </si>
+  <si>
+    <t>Gwydr aildoddi</t>
+  </si>
+  <si>
+    <t>prns.list.filter.paper</t>
+  </si>
+  <si>
+    <t>Paper, board or fibre-based composite material</t>
+  </si>
+  <si>
+    <t>Papur, bwrdd neu ddeunydd cyfansawdd sy'n seiliedig ar ffeibrau</t>
+  </si>
+  <si>
+    <t>prns.list.filter.plastic</t>
+  </si>
+  <si>
+    <t>Plastic</t>
+  </si>
+  <si>
+    <t>Plastig</t>
+  </si>
+  <si>
+    <t>prns.list.filter.steel</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>Dur</t>
+  </si>
+  <si>
+    <t>prns.list.filter.wood</t>
+  </si>
+  <si>
+    <t>Wood</t>
+  </si>
+  <si>
+    <t>Pren</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.landmark</t>
+  </si>
+  <si>
+    <t>results</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.previous</t>
+  </si>
+  <si>
+    <t>Previous</t>
+  </si>
+  <si>
+    <t>Blaenorol</t>
+  </si>
+  <si>
+    <t>prns.list.pagination.next</t>
+  </si>
+  <si>
+    <t>Next</t>
+  </si>
+  <si>
+    <t>Nesaf</t>
   </si>
 </sst>
 </file>
@@ -556,7 +748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -627,7 +819,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -647,7 +839,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -861,7 +1053,7 @@
         <v>39</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>13</v>
@@ -869,7 +1061,7 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>10</v>
@@ -878,10 +1070,10 @@
         <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>13</v>
@@ -889,7 +1081,7 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>10</v>
@@ -898,10 +1090,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>13</v>
@@ -909,7 +1101,7 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>10</v>
@@ -918,10 +1110,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
@@ -929,7 +1121,7 @@
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>10</v>
@@ -938,17 +1130,477 @@
         <v>11</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F22"/>
+  <autoFilter ref="A5:F45"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
MO-478: Add DW flash to Accept/Reject page
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
+++ b/translations/welsh-translations/xlsx/15-producer-prns-list.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="115">
   <si>
     <t>Translator notes</t>
   </si>
@@ -110,6 +110,12 @@
   </si>
   <si>
     <t>Select {{number}}</t>
+  </si>
+  <si>
+    <t>prns.list.decemberWasteFlash</t>
+  </si>
+  <si>
+    <t>Can be accepted towards {{firstYear}} or {{secondYear}}</t>
   </si>
   <si>
     <t>prns.list.tableCaption</t>
@@ -748,7 +754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1033,7 +1039,7 @@
         <v>36</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>13</v>
@@ -1041,19 +1047,19 @@
     </row>
     <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>13</v>
@@ -1061,19 +1067,19 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>13</v>
@@ -1081,19 +1087,19 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>13</v>
@@ -1101,19 +1107,19 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
@@ -1133,7 +1139,7 @@
         <v>50</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>13</v>
@@ -1141,19 +1147,19 @@
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>13</v>
@@ -1213,7 +1219,7 @@
         <v>59</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>13</v>
@@ -1221,19 +1227,19 @@
     </row>
     <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="1" t="s">
+      <c r="E27" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>13</v>
@@ -1273,7 +1279,7 @@
         <v>66</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>13</v>
@@ -1281,19 +1287,19 @@
     </row>
     <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="1" t="s">
+      <c r="E30" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>13</v>
@@ -1301,19 +1307,19 @@
     </row>
     <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>13</v>
@@ -1353,7 +1359,7 @@
         <v>76</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>77</v>
+        <v>13</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>13</v>
@@ -1361,19 +1367,19 @@
     </row>
     <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>13</v>
@@ -1381,19 +1387,19 @@
     </row>
     <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="1" t="s">
+      <c r="E35" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>13</v>
@@ -1401,19 +1407,19 @@
     </row>
     <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="1" t="s">
+      <c r="E36" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>86</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>13</v>
@@ -1421,19 +1427,19 @@
     </row>
     <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>13</v>
@@ -1441,19 +1447,19 @@
     </row>
     <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D38" s="1" t="s">
+      <c r="E38" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>13</v>
@@ -1461,19 +1467,19 @@
     </row>
     <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D39" s="1" t="s">
+      <c r="E39" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>13</v>
@@ -1481,19 +1487,19 @@
     </row>
     <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D40" s="1" t="s">
+      <c r="E40" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>13</v>
@@ -1501,19 +1507,19 @@
     </row>
     <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="1" t="s">
+      <c r="E41" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>13</v>
@@ -1521,19 +1527,19 @@
     </row>
     <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D42" s="1" t="s">
+      <c r="E42" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>13</v>
@@ -1541,19 +1547,19 @@
     </row>
     <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D43" s="1" t="s">
+      <c r="E43" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>13</v>
@@ -1573,7 +1579,7 @@
         <v>108</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>109</v>
+        <v>13</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>13</v>
@@ -1581,26 +1587,46 @@
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="F45" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="B46" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F45"/>
+  <autoFilter ref="A5:F46"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>